<commit_message>
Série A: 14 nomes vetados pelo clube (titulares, negociados); listas regeradas
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EuPBN7B2QoMn8WDwKax4KN
</commit_message>
<xml_diff>
--- a/Santa Cruz V2/listas/listas_2027.xlsx
+++ b/Santa Cruz V2/listas/listas_2027.xlsx
@@ -958,9 +958,6 @@
     <t>David Duarte</t>
   </si>
   <si>
-    <t>Ignácio</t>
-  </si>
-  <si>
     <t>Fabricio Bruno</t>
   </si>
   <si>
@@ -976,6 +973,9 @@
     <t>João Victor</t>
   </si>
   <si>
+    <t>Tiago Cóser</t>
+  </si>
+  <si>
     <t>Viery</t>
   </si>
   <si>
@@ -1084,15 +1084,9 @@
     <t>A. Montoro</t>
   </si>
   <si>
-    <t>Negueba</t>
-  </si>
-  <si>
     <t>Keny Arroyo</t>
   </si>
   <si>
-    <t>J. Carrascal</t>
-  </si>
-  <si>
     <t>Erick</t>
   </si>
   <si>
@@ -1108,6 +1102,12 @@
     <t>Gabriel Bontempo</t>
   </si>
   <si>
+    <t>J. Herrera</t>
+  </si>
+  <si>
+    <t>Nuno Moreira</t>
+  </si>
+  <si>
     <t>Samuel Lino</t>
   </si>
   <si>
@@ -1186,21 +1186,21 @@
     <t>Flamengo</t>
   </si>
   <si>
+    <t>Cruzeiro</t>
+  </si>
+  <si>
+    <t>Corinthians</t>
+  </si>
+  <si>
+    <t>Mirassol</t>
+  </si>
+  <si>
+    <t>Grêmio</t>
+  </si>
+  <si>
     <t>Fluminense</t>
   </si>
   <si>
-    <t>Cruzeiro</t>
-  </si>
-  <si>
-    <t>Corinthians</t>
-  </si>
-  <si>
-    <t>Mirassol</t>
-  </si>
-  <si>
-    <t>Grêmio</t>
-  </si>
-  <si>
     <t>Chapecoense</t>
   </si>
   <si>
@@ -1213,19 +1213,19 @@
     <t>2030-12-31</t>
   </si>
   <si>
+    <t>2031-06-30</t>
+  </si>
+  <si>
+    <t>2029-06-30</t>
+  </si>
+  <si>
+    <t>2027-04-10</t>
+  </si>
+  <si>
+    <t>2031-01-31</t>
+  </si>
+  <si>
     <t>2028-06-30</t>
-  </si>
-  <si>
-    <t>2031-06-30</t>
-  </si>
-  <si>
-    <t>2029-06-30</t>
-  </si>
-  <si>
-    <t>2027-04-10</t>
-  </si>
-  <si>
-    <t>2031-01-31</t>
   </si>
   <si>
     <t>Uruguay</t>
@@ -24091,16 +24091,16 @@
         <v>388</v>
       </c>
       <c r="F20">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G20">
-        <v>920</v>
+        <v>2013</v>
       </c>
       <c r="H20" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="I20">
-        <v>1500000</v>
+        <v>0</v>
       </c>
       <c r="J20" t="s">
         <v>272</v>
@@ -24109,19 +24109,19 @@
         <v>272</v>
       </c>
       <c r="L20">
-        <v>58.3</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="M20">
-        <v>64.3</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="N20">
-        <v>58.9</v>
+        <v>52.4</v>
       </c>
       <c r="O20">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="P20">
-        <v>61.6</v>
+        <v>60.9</v>
       </c>
       <c r="Q20" t="b">
         <v>1</v>
@@ -24130,22 +24130,22 @@
         <v>0</v>
       </c>
       <c r="S20">
-        <v>30.9</v>
+        <v>28.4</v>
       </c>
       <c r="T20">
         <v>7</v>
       </c>
       <c r="U20">
-        <v>60</v>
+        <v>56.7</v>
       </c>
       <c r="V20">
-        <v>5.1</v>
+        <v>3.7</v>
       </c>
       <c r="W20">
-        <v>5</v>
+        <v>4.1</v>
       </c>
       <c r="X20">
-        <v>1.7</v>
+        <v>0.3</v>
       </c>
       <c r="Y20" t="b">
         <v>1</v>
@@ -24180,19 +24180,19 @@
         <v>313</v>
       </c>
       <c r="E21" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="F21">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G21">
-        <v>2013</v>
+        <v>1620</v>
       </c>
       <c r="H21" t="s">
-        <v>396</v>
+        <v>261</v>
       </c>
       <c r="I21">
-        <v>0</v>
+        <v>1000000</v>
       </c>
       <c r="J21" t="s">
         <v>272</v>
@@ -24201,19 +24201,19 @@
         <v>272</v>
       </c>
       <c r="L21">
-        <v>76.40000000000001</v>
+        <v>59.4</v>
       </c>
       <c r="M21">
-        <v>69.40000000000001</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="N21">
-        <v>52.4</v>
+        <v>53.3</v>
       </c>
       <c r="O21">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="P21">
-        <v>60.9</v>
+        <v>59</v>
       </c>
       <c r="Q21" t="b">
         <v>1</v>
@@ -24222,22 +24222,22 @@
         <v>0</v>
       </c>
       <c r="S21">
-        <v>28.4</v>
+        <v>36.2</v>
       </c>
       <c r="T21">
         <v>7</v>
       </c>
       <c r="U21">
-        <v>56.7</v>
+        <v>45.2</v>
       </c>
       <c r="V21">
-        <v>3.7</v>
+        <v>4.6</v>
       </c>
       <c r="W21">
-        <v>4.1</v>
+        <v>3</v>
       </c>
       <c r="X21">
-        <v>0.3</v>
+        <v>1.9</v>
       </c>
       <c r="Y21" t="b">
         <v>1</v>
@@ -24272,40 +24272,40 @@
         <v>314</v>
       </c>
       <c r="E22" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="F22">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G22">
-        <v>1620</v>
+        <v>1078</v>
       </c>
       <c r="H22" t="s">
         <v>261</v>
       </c>
       <c r="I22">
-        <v>1000000</v>
+        <v>0</v>
       </c>
       <c r="J22" t="s">
-        <v>272</v>
+        <v>402</v>
       </c>
       <c r="K22" t="s">
-        <v>272</v>
+        <v>402</v>
       </c>
       <c r="L22">
-        <v>59.4</v>
+        <v>48.6</v>
       </c>
       <c r="M22">
-        <v>64.59999999999999</v>
+        <v>61.6</v>
       </c>
       <c r="N22">
-        <v>53.3</v>
+        <v>54.5</v>
       </c>
       <c r="O22">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="P22">
-        <v>59</v>
+        <v>58.1</v>
       </c>
       <c r="Q22" t="b">
         <v>1</v>
@@ -24314,19 +24314,19 @@
         <v>0</v>
       </c>
       <c r="S22">
-        <v>36.2</v>
+        <v>29.1</v>
       </c>
       <c r="T22">
         <v>7</v>
       </c>
       <c r="U22">
-        <v>45.2</v>
+        <v>56.2</v>
       </c>
       <c r="V22">
-        <v>4.6</v>
+        <v>5.9</v>
       </c>
       <c r="W22">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="X22">
         <v>1.9</v>
@@ -24335,7 +24335,7 @@
         <v>1</v>
       </c>
       <c r="Z22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA22" t="s">
         <v>284</v>
@@ -24347,7 +24347,7 @@
         <v>0</v>
       </c>
       <c r="AD22" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="23" spans="1:30">
@@ -24364,40 +24364,40 @@
         <v>315</v>
       </c>
       <c r="E23" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="F23">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="G23">
-        <v>1078</v>
+        <v>1810</v>
       </c>
       <c r="H23" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="I23">
-        <v>0</v>
+        <v>2000000</v>
       </c>
       <c r="J23" t="s">
-        <v>402</v>
+        <v>272</v>
       </c>
       <c r="K23" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="L23">
-        <v>48.6</v>
+        <v>58.5</v>
       </c>
       <c r="M23">
-        <v>61.6</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="N23">
-        <v>54.5</v>
+        <v>48.9</v>
       </c>
       <c r="O23">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="P23">
-        <v>58.1</v>
+        <v>56.7</v>
       </c>
       <c r="Q23" t="b">
         <v>1</v>
@@ -24406,28 +24406,28 @@
         <v>0</v>
       </c>
       <c r="S23">
-        <v>29.1</v>
+        <v>32.9</v>
       </c>
       <c r="T23">
         <v>7</v>
       </c>
       <c r="U23">
-        <v>56.2</v>
+        <v>51</v>
       </c>
       <c r="V23">
-        <v>5.9</v>
+        <v>2.9</v>
       </c>
       <c r="W23">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="X23">
-        <v>1.9</v>
+        <v>0.3</v>
       </c>
       <c r="Y23" t="b">
         <v>1</v>
       </c>
       <c r="Z23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA23" t="s">
         <v>284</v>
@@ -24439,7 +24439,7 @@
         <v>0</v>
       </c>
       <c r="AD23" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="24" spans="1:30">
@@ -24459,37 +24459,37 @@
         <v>390</v>
       </c>
       <c r="F24">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="G24">
-        <v>1810</v>
+        <v>2261</v>
       </c>
       <c r="H24" t="s">
         <v>256</v>
       </c>
       <c r="I24">
-        <v>2000000</v>
+        <v>250000</v>
       </c>
       <c r="J24" t="s">
         <v>272</v>
       </c>
       <c r="K24" t="s">
-        <v>407</v>
+        <v>272</v>
       </c>
       <c r="L24">
-        <v>58.5</v>
+        <v>54.3</v>
       </c>
       <c r="M24">
-        <v>64.40000000000001</v>
+        <v>63.2</v>
       </c>
       <c r="N24">
-        <v>48.9</v>
+        <v>50</v>
       </c>
       <c r="O24">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P24">
-        <v>56.7</v>
+        <v>56.6</v>
       </c>
       <c r="Q24" t="b">
         <v>1</v>
@@ -24498,22 +24498,22 @@
         <v>0</v>
       </c>
       <c r="S24">
-        <v>32.9</v>
+        <v>28.6</v>
       </c>
       <c r="T24">
         <v>7</v>
       </c>
       <c r="U24">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="V24">
         <v>2.9</v>
       </c>
       <c r="W24">
-        <v>3</v>
+        <v>4.6</v>
       </c>
       <c r="X24">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="Y24" t="b">
         <v>1</v>
@@ -24548,40 +24548,40 @@
         <v>317</v>
       </c>
       <c r="E25" t="s">
-        <v>391</v>
+        <v>381</v>
       </c>
       <c r="F25">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="G25">
-        <v>2261</v>
+        <v>1549</v>
       </c>
       <c r="H25" t="s">
         <v>256</v>
       </c>
       <c r="I25">
-        <v>250000</v>
+        <v>400000</v>
       </c>
       <c r="J25" t="s">
         <v>272</v>
       </c>
       <c r="K25" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="L25">
-        <v>54.3</v>
+        <v>50.9</v>
       </c>
       <c r="M25">
-        <v>63.2</v>
+        <v>62.3</v>
       </c>
       <c r="N25">
-        <v>50</v>
+        <v>48.5</v>
       </c>
       <c r="O25">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="P25">
-        <v>56.6</v>
+        <v>55.4</v>
       </c>
       <c r="Q25" t="b">
         <v>1</v>
@@ -24590,22 +24590,22 @@
         <v>0</v>
       </c>
       <c r="S25">
-        <v>28.6</v>
+        <v>29.2</v>
       </c>
       <c r="T25">
         <v>7</v>
       </c>
       <c r="U25">
-        <v>54</v>
+        <v>39.5</v>
       </c>
       <c r="V25">
-        <v>2.9</v>
+        <v>3.7</v>
       </c>
       <c r="W25">
-        <v>4.6</v>
+        <v>2.7</v>
       </c>
       <c r="X25">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="Y25" t="b">
         <v>1</v>
@@ -24623,7 +24623,7 @@
         <v>0</v>
       </c>
       <c r="AD25" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="26" spans="1:30">
@@ -24640,7 +24640,7 @@
         <v>318</v>
       </c>
       <c r="E26" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F26">
         <v>21</v>
@@ -24649,7 +24649,7 @@
         <v>1323</v>
       </c>
       <c r="H26" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="I26">
         <v>0</v>
@@ -24824,7 +24824,7 @@
         <v>320</v>
       </c>
       <c r="E28" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="F28">
         <v>26</v>
@@ -25008,7 +25008,7 @@
         <v>322</v>
       </c>
       <c r="E30" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="F30">
         <v>29</v>
@@ -25100,7 +25100,7 @@
         <v>323</v>
       </c>
       <c r="E31" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F31">
         <v>22</v>
@@ -25109,7 +25109,7 @@
         <v>1411</v>
       </c>
       <c r="H31" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I31">
         <v>0</v>
@@ -25560,7 +25560,7 @@
         <v>328</v>
       </c>
       <c r="E36" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="F36">
         <v>27</v>
@@ -25744,7 +25744,7 @@
         <v>330</v>
       </c>
       <c r="E38" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F38">
         <v>23</v>
@@ -25836,7 +25836,7 @@
         <v>331</v>
       </c>
       <c r="E39" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="F39">
         <v>33</v>
@@ -25928,7 +25928,7 @@
         <v>332</v>
       </c>
       <c r="E40" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="F40">
         <v>29</v>
@@ -26112,7 +26112,7 @@
         <v>334</v>
       </c>
       <c r="E42" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="F42">
         <v>28</v>
@@ -26204,7 +26204,7 @@
         <v>335</v>
       </c>
       <c r="E43" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="F43">
         <v>24</v>
@@ -26388,7 +26388,7 @@
         <v>336</v>
       </c>
       <c r="E45" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F45">
         <v>24</v>
@@ -26581,7 +26581,7 @@
         <v>1133</v>
       </c>
       <c r="H47" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="I47">
         <v>0</v>
@@ -26652,7 +26652,7 @@
         <v>338</v>
       </c>
       <c r="E48" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="F48">
         <v>25</v>
@@ -26744,7 +26744,7 @@
         <v>339</v>
       </c>
       <c r="E49" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F49">
         <v>29</v>
@@ -26925,7 +26925,7 @@
         <v>1495</v>
       </c>
       <c r="H51" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I51">
         <v>0</v>
@@ -27640,7 +27640,7 @@
         <v>348</v>
       </c>
       <c r="E59" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="F59">
         <v>32</v>
@@ -27732,7 +27732,7 @@
         <v>349</v>
       </c>
       <c r="E60" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F60">
         <v>30</v>
@@ -27916,7 +27916,7 @@
         <v>351</v>
       </c>
       <c r="E62" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="F62">
         <v>28</v>
@@ -28284,40 +28284,40 @@
         <v>354</v>
       </c>
       <c r="E66" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="F66">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G66">
-        <v>907</v>
+        <v>1196</v>
       </c>
       <c r="H66" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I66">
-        <v>450000</v>
+        <v>0</v>
       </c>
       <c r="J66" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="K66" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="L66">
-        <v>67.3</v>
+        <v>63.2</v>
       </c>
       <c r="M66">
-        <v>66.8</v>
+        <v>65.7</v>
       </c>
       <c r="N66">
-        <v>58.6</v>
+        <v>55.4</v>
       </c>
       <c r="O66">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P66">
-        <v>62.7</v>
+        <v>60.6</v>
       </c>
       <c r="Q66" t="b">
         <v>1</v>
@@ -28326,28 +28326,28 @@
         <v>0</v>
       </c>
       <c r="S66">
-        <v>38.9</v>
+        <v>48.9</v>
       </c>
       <c r="T66">
         <v>6</v>
       </c>
       <c r="U66">
-        <v>54</v>
+        <v>56.7</v>
       </c>
       <c r="V66">
-        <v>3.6</v>
+        <v>4.5</v>
       </c>
       <c r="W66">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="X66">
-        <v>9.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="Y66" t="b">
         <v>1</v>
       </c>
       <c r="Z66" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA66" t="s">
         <v>284</v>
@@ -28359,7 +28359,7 @@
         <v>0</v>
       </c>
       <c r="AD66" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="67" spans="1:30">
@@ -28376,40 +28376,40 @@
         <v>355</v>
       </c>
       <c r="E67" t="s">
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="F67">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G67">
-        <v>1196</v>
+        <v>1691</v>
       </c>
       <c r="H67" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="I67">
-        <v>0</v>
+        <v>1200000</v>
       </c>
       <c r="J67" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="K67" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="L67">
-        <v>63.2</v>
+        <v>34.1</v>
       </c>
       <c r="M67">
-        <v>65.7</v>
+        <v>57.5</v>
       </c>
       <c r="N67">
-        <v>55.4</v>
+        <v>58.5</v>
       </c>
       <c r="O67">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P67">
-        <v>60.6</v>
+        <v>58</v>
       </c>
       <c r="Q67" t="b">
         <v>1</v>
@@ -28418,28 +28418,28 @@
         <v>0</v>
       </c>
       <c r="S67">
-        <v>48.9</v>
+        <v>32.6</v>
       </c>
       <c r="T67">
         <v>6</v>
       </c>
       <c r="U67">
-        <v>56.7</v>
+        <v>43.4</v>
       </c>
       <c r="V67">
-        <v>4.5</v>
+        <v>3.1</v>
       </c>
       <c r="W67">
-        <v>1.8</v>
+        <v>0.6</v>
       </c>
       <c r="X67">
-        <v>7.8</v>
+        <v>10.1</v>
       </c>
       <c r="Y67" t="b">
         <v>1</v>
       </c>
       <c r="Z67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA67" t="s">
         <v>284</v>
@@ -28451,7 +28451,7 @@
         <v>0</v>
       </c>
       <c r="AD67" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="68" spans="1:30">
@@ -28468,58 +28468,70 @@
         <v>356</v>
       </c>
       <c r="E68" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="F68">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G68">
-        <v>957</v>
+        <v>1579</v>
       </c>
       <c r="H68" t="s">
-        <v>399</v>
+        <v>256</v>
       </c>
       <c r="I68">
         <v>0</v>
       </c>
       <c r="J68" t="s">
-        <v>403</v>
+        <v>272</v>
       </c>
       <c r="K68" t="s">
-        <v>403</v>
+        <v>272</v>
       </c>
       <c r="L68">
-        <v>72.7</v>
+        <v>63.4</v>
       </c>
       <c r="M68">
-        <v>68.40000000000001</v>
+        <v>65.8</v>
+      </c>
+      <c r="N68">
+        <v>50.1</v>
+      </c>
+      <c r="O68">
+        <v>13</v>
       </c>
       <c r="P68">
-        <v>59.6</v>
+        <v>58</v>
       </c>
       <c r="Q68" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="R68">
+        <v>0</v>
+      </c>
+      <c r="S68">
+        <v>45</v>
       </c>
       <c r="T68">
         <v>6</v>
       </c>
       <c r="U68">
-        <v>67</v>
+        <v>39.5</v>
       </c>
       <c r="V68">
-        <v>7.1</v>
+        <v>5.2</v>
       </c>
       <c r="W68">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="X68">
-        <v>7</v>
+        <v>14.7</v>
       </c>
       <c r="Y68" t="b">
         <v>1</v>
       </c>
       <c r="Z68" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA68" t="s">
         <v>284</v>
@@ -28531,7 +28543,7 @@
         <v>0</v>
       </c>
       <c r="AD68" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="69" spans="1:30">
@@ -28548,19 +28560,19 @@
         <v>357</v>
       </c>
       <c r="E69" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="F69">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="G69">
-        <v>1691</v>
+        <v>1605</v>
       </c>
       <c r="H69" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="I69">
-        <v>1200000</v>
+        <v>0</v>
       </c>
       <c r="J69" t="s">
         <v>272</v>
@@ -28569,19 +28581,19 @@
         <v>272</v>
       </c>
       <c r="L69">
-        <v>34.1</v>
+        <v>48.6</v>
       </c>
       <c r="M69">
-        <v>57.5</v>
+        <v>61.6</v>
       </c>
       <c r="N69">
-        <v>58.5</v>
+        <v>51.6</v>
       </c>
       <c r="O69">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="P69">
-        <v>58</v>
+        <v>56.6</v>
       </c>
       <c r="Q69" t="b">
         <v>1</v>
@@ -28590,22 +28602,22 @@
         <v>0</v>
       </c>
       <c r="S69">
-        <v>32.6</v>
+        <v>43.9</v>
       </c>
       <c r="T69">
         <v>6</v>
       </c>
       <c r="U69">
-        <v>43.4</v>
+        <v>52.4</v>
       </c>
       <c r="V69">
-        <v>3.1</v>
+        <v>5.9</v>
       </c>
       <c r="W69">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="X69">
-        <v>10.1</v>
+        <v>11.8</v>
       </c>
       <c r="Y69" t="b">
         <v>1</v>
@@ -28623,7 +28635,7 @@
         <v>0</v>
       </c>
       <c r="AD69" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="70" spans="1:30">
@@ -28640,16 +28652,16 @@
         <v>358</v>
       </c>
       <c r="E70" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="F70">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="G70">
-        <v>1579</v>
+        <v>1029</v>
       </c>
       <c r="H70" t="s">
-        <v>256</v>
+        <v>396</v>
       </c>
       <c r="I70">
         <v>0</v>
@@ -28658,46 +28670,34 @@
         <v>272</v>
       </c>
       <c r="K70" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="L70">
-        <v>63.4</v>
+        <v>45.9</v>
       </c>
       <c r="M70">
-        <v>65.8</v>
-      </c>
-      <c r="N70">
-        <v>50.1</v>
-      </c>
-      <c r="O70">
-        <v>13</v>
+        <v>60.9</v>
       </c>
       <c r="P70">
-        <v>58</v>
+        <v>55.9</v>
       </c>
       <c r="Q70" t="b">
-        <v>1</v>
-      </c>
-      <c r="R70">
-        <v>0</v>
-      </c>
-      <c r="S70">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="T70">
         <v>6</v>
       </c>
       <c r="U70">
-        <v>39.5</v>
+        <v>67</v>
       </c>
       <c r="V70">
-        <v>5.2</v>
+        <v>10.5</v>
       </c>
       <c r="W70">
-        <v>2.2</v>
+        <v>4</v>
       </c>
       <c r="X70">
-        <v>14.7</v>
+        <v>8</v>
       </c>
       <c r="Y70" t="b">
         <v>1</v>
@@ -28715,7 +28715,7 @@
         <v>0</v>
       </c>
       <c r="AD70" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="71" spans="1:30">
@@ -28732,16 +28732,16 @@
         <v>359</v>
       </c>
       <c r="E71" t="s">
-        <v>386</v>
+        <v>297</v>
       </c>
       <c r="F71">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G71">
-        <v>1605</v>
+        <v>1392</v>
       </c>
       <c r="H71" t="s">
-        <v>257</v>
+        <v>396</v>
       </c>
       <c r="I71">
         <v>0</v>
@@ -28753,19 +28753,19 @@
         <v>272</v>
       </c>
       <c r="L71">
-        <v>48.6</v>
+        <v>66.8</v>
       </c>
       <c r="M71">
-        <v>61.6</v>
+        <v>66.7</v>
       </c>
       <c r="N71">
-        <v>51.6</v>
+        <v>45</v>
       </c>
       <c r="O71">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="P71">
-        <v>56.6</v>
+        <v>55.8</v>
       </c>
       <c r="Q71" t="b">
         <v>1</v>
@@ -28774,22 +28774,22 @@
         <v>0</v>
       </c>
       <c r="S71">
-        <v>43.9</v>
+        <v>37.3</v>
       </c>
       <c r="T71">
         <v>6</v>
       </c>
       <c r="U71">
-        <v>52.4</v>
+        <v>48.4</v>
       </c>
       <c r="V71">
-        <v>5.9</v>
+        <v>3.8</v>
       </c>
       <c r="W71">
-        <v>0.9</v>
+        <v>1.7</v>
       </c>
       <c r="X71">
-        <v>11.8</v>
+        <v>5.5</v>
       </c>
       <c r="Y71" t="b">
         <v>1</v>
@@ -28824,58 +28824,70 @@
         <v>360</v>
       </c>
       <c r="E72" t="s">
-        <v>387</v>
+        <v>378</v>
       </c>
       <c r="F72">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G72">
-        <v>1029</v>
+        <v>1039</v>
       </c>
       <c r="H72" t="s">
-        <v>396</v>
+        <v>257</v>
       </c>
       <c r="I72">
         <v>0</v>
       </c>
       <c r="J72" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="K72" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="L72">
-        <v>45.9</v>
+        <v>62.7</v>
       </c>
       <c r="M72">
-        <v>60.9</v>
+        <v>65.59999999999999</v>
+      </c>
+      <c r="N72">
+        <v>43.8</v>
+      </c>
+      <c r="O72">
+        <v>17</v>
       </c>
       <c r="P72">
-        <v>55.9</v>
+        <v>54.7</v>
       </c>
       <c r="Q72" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="R72">
+        <v>0</v>
+      </c>
+      <c r="S72">
+        <v>43.5</v>
       </c>
       <c r="T72">
         <v>6</v>
       </c>
       <c r="U72">
-        <v>67</v>
+        <v>45.2</v>
       </c>
       <c r="V72">
-        <v>10.5</v>
+        <v>5.6</v>
       </c>
       <c r="W72">
-        <v>4</v>
+        <v>2.2</v>
       </c>
       <c r="X72">
-        <v>8</v>
+        <v>7.6</v>
       </c>
       <c r="Y72" t="b">
         <v>1</v>
       </c>
       <c r="Z72" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA72" t="s">
         <v>284</v>
@@ -28887,7 +28899,7 @@
         <v>0</v>
       </c>
       <c r="AD72" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="73" spans="1:30">
@@ -28904,40 +28916,40 @@
         <v>361</v>
       </c>
       <c r="E73" t="s">
-        <v>297</v>
+        <v>384</v>
       </c>
       <c r="F73">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="G73">
-        <v>1392</v>
+        <v>1005</v>
       </c>
       <c r="H73" t="s">
-        <v>396</v>
+        <v>256</v>
       </c>
       <c r="I73">
-        <v>0</v>
+        <v>1000000</v>
       </c>
       <c r="J73" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K73" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="L73">
-        <v>66.8</v>
+        <v>34.5</v>
       </c>
       <c r="M73">
-        <v>66.7</v>
+        <v>57.7</v>
       </c>
       <c r="N73">
-        <v>45</v>
+        <v>50.2</v>
       </c>
       <c r="O73">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="P73">
-        <v>55.8</v>
+        <v>53.9</v>
       </c>
       <c r="Q73" t="b">
         <v>1</v>
@@ -28946,28 +28958,28 @@
         <v>0</v>
       </c>
       <c r="S73">
-        <v>37.3</v>
+        <v>36.9</v>
       </c>
       <c r="T73">
         <v>6</v>
       </c>
       <c r="U73">
-        <v>48.4</v>
+        <v>56.2</v>
       </c>
       <c r="V73">
-        <v>3.8</v>
+        <v>4.6</v>
       </c>
       <c r="W73">
-        <v>1.7</v>
+        <v>1.2</v>
       </c>
       <c r="X73">
-        <v>5.5</v>
+        <v>4.8</v>
       </c>
       <c r="Y73" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA73" t="s">
         <v>284</v>
@@ -28979,7 +28991,7 @@
         <v>0</v>
       </c>
       <c r="AD73" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="74" spans="1:30">
@@ -29097,7 +29109,7 @@
         <v>1715</v>
       </c>
       <c r="H75" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="I75">
         <v>0</v>
@@ -29364,7 +29376,7 @@
         <v>366</v>
       </c>
       <c r="E78" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="F78">
         <v>28</v>
@@ -29456,7 +29468,7 @@
         <v>367</v>
       </c>
       <c r="E79" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="F79">
         <v>27</v>
@@ -29925,7 +29937,7 @@
         <v>2216</v>
       </c>
       <c r="H84" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I84">
         <v>0</v>
@@ -30100,7 +30112,7 @@
         <v>374</v>
       </c>
       <c r="E86" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F86">
         <v>24</v>
@@ -31721,7 +31733,7 @@
         <v>1599</v>
       </c>
       <c r="H15" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I15">
         <v>450000</v>
@@ -34059,7 +34071,7 @@
         <v>1213</v>
       </c>
       <c r="H41" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I41">
         <v>0</v>
@@ -34964,7 +34976,7 @@
         <v>1700</v>
       </c>
       <c r="H51" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="I51">
         <v>0</v>
@@ -39471,7 +39483,7 @@
         <v>1626</v>
       </c>
       <c r="H101" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I101">
         <v>0</v>
@@ -40818,7 +40830,7 @@
         <v>1341</v>
       </c>
       <c r="H116" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I116">
         <v>0</v>
@@ -41079,7 +41091,7 @@
         <v>1507</v>
       </c>
       <c r="H119" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I119">
         <v>325000</v>
@@ -41447,7 +41459,7 @@
         <v>1393</v>
       </c>
       <c r="H123" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I123">
         <v>0</v>
@@ -43083,7 +43095,7 @@
         <v>3387</v>
       </c>
       <c r="H8" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I8">
         <v>350000</v>
@@ -43261,7 +43273,7 @@
         <v>4420</v>
       </c>
       <c r="H10" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I10">
         <v>300000</v>
@@ -43525,7 +43537,7 @@
         <v>2240</v>
       </c>
       <c r="H13" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -43614,7 +43626,7 @@
         <v>1162</v>
       </c>
       <c r="H14" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I14">
         <v>2000000</v>
@@ -44427,7 +44439,7 @@
         <v>3017</v>
       </c>
       <c r="H23" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I23">
         <v>125000</v>
@@ -44516,7 +44528,7 @@
         <v>2596</v>
       </c>
       <c r="H24" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I24">
         <v>1000000</v>
@@ -44878,7 +44890,7 @@
         <v>3268</v>
       </c>
       <c r="H28" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I28">
         <v>250000</v>
@@ -45044,7 +45056,7 @@
         <v>6</v>
       </c>
       <c r="D30" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E30" t="s">
         <v>845</v>
@@ -45148,7 +45160,7 @@
         <v>2644</v>
       </c>
       <c r="H31" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I31">
         <v>800000</v>
@@ -45424,7 +45436,7 @@
         <v>1336</v>
       </c>
       <c r="H34" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I34">
         <v>300000</v>
@@ -45694,7 +45706,7 @@
         <v>4311</v>
       </c>
       <c r="H37" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I37">
         <v>0</v>
@@ -45786,7 +45798,7 @@
         <v>1834</v>
       </c>
       <c r="H38" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I38">
         <v>800000</v>
@@ -45967,7 +45979,7 @@
         <v>3128</v>
       </c>
       <c r="H40" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I40">
         <v>0</v>
@@ -46059,7 +46071,7 @@
         <v>1775</v>
       </c>
       <c r="H41" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I41">
         <v>250000</v>
@@ -46148,7 +46160,7 @@
         <v>3055</v>
       </c>
       <c r="H42" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I42">
         <v>500000</v>
@@ -46418,7 +46430,7 @@
         <v>2070</v>
       </c>
       <c r="H45" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I45">
         <v>500000</v>
@@ -46869,7 +46881,7 @@
         <v>2048</v>
       </c>
       <c r="H50" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="I50">
         <v>0</v>
@@ -47587,7 +47599,7 @@
         <v>1600</v>
       </c>
       <c r="H58" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I58">
         <v>0</v>
@@ -47762,7 +47774,7 @@
         <v>1730</v>
       </c>
       <c r="H60" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I60">
         <v>0</v>
@@ -48391,7 +48403,7 @@
         <v>3101</v>
       </c>
       <c r="H67" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I67">
         <v>0</v>
@@ -48750,7 +48762,7 @@
         <v>2806</v>
       </c>
       <c r="H71" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I71">
         <v>1000000</v>
@@ -49385,7 +49397,7 @@
         <v>2482</v>
       </c>
       <c r="H78" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I78">
         <v>1200000</v>
@@ -49928,7 +49940,7 @@
         <v>901</v>
       </c>
       <c r="H84" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I84">
         <v>0</v>
@@ -50017,7 +50029,7 @@
         <v>2203</v>
       </c>
       <c r="H85" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I85">
         <v>0</v>
@@ -50557,7 +50569,7 @@
         <v>2179</v>
       </c>
       <c r="H91" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I91">
         <v>1000000</v>
@@ -51103,7 +51115,7 @@
         <v>2760</v>
       </c>
       <c r="H97" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I97">
         <v>300000</v>
@@ -51192,7 +51204,7 @@
         <v>1531</v>
       </c>
       <c r="H98" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I98">
         <v>0</v>
@@ -51548,7 +51560,7 @@
         <v>1910</v>
       </c>
       <c r="H102" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I102">
         <v>0</v>
@@ -52082,7 +52094,7 @@
         <v>3542</v>
       </c>
       <c r="H108" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I108">
         <v>0</v>
@@ -52174,7 +52186,7 @@
         <v>1570</v>
       </c>
       <c r="H109" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I109">
         <v>200000</v>
@@ -52266,7 +52278,7 @@
         <v>1774</v>
       </c>
       <c r="H110" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I110">
         <v>1000000</v>
@@ -52358,7 +52370,7 @@
         <v>2761</v>
       </c>
       <c r="H111" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I111">
         <v>0</v>
@@ -52450,7 +52462,7 @@
         <v>2669</v>
       </c>
       <c r="H112" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I112">
         <v>0</v>
@@ -52809,7 +52821,7 @@
         <v>2691</v>
       </c>
       <c r="H116" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I116">
         <v>0</v>
@@ -53174,7 +53186,7 @@
         <v>1605</v>
       </c>
       <c r="H120" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I120">
         <v>600000</v>
@@ -53352,7 +53364,7 @@
         <v>1543</v>
       </c>
       <c r="H122" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I122">
         <v>0</v>
@@ -53533,7 +53545,7 @@
         <v>1804</v>
       </c>
       <c r="H124" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I124">
         <v>700000</v>
@@ -54890,7 +54902,7 @@
         <v>3693</v>
       </c>
       <c r="H6" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I6">
         <v>1500000</v>
@@ -55154,7 +55166,7 @@
         <v>3042</v>
       </c>
       <c r="H9" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I9">
         <v>300000</v>
@@ -55510,7 +55522,7 @@
         <v>2219</v>
       </c>
       <c r="H13" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I13">
         <v>400000</v>
@@ -55777,7 +55789,7 @@
         <v>1052</v>
       </c>
       <c r="H16" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I16">
         <v>0</v>
@@ -55866,7 +55878,7 @@
         <v>1491</v>
       </c>
       <c r="H17" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I17">
         <v>400000</v>
@@ -56047,7 +56059,7 @@
         <v>2458</v>
       </c>
       <c r="H19" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I19">
         <v>0</v>
@@ -56139,7 +56151,7 @@
         <v>2545</v>
       </c>
       <c r="H20" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I20">
         <v>0</v>
@@ -56228,7 +56240,7 @@
         <v>3339</v>
       </c>
       <c r="H21" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I21">
         <v>500000</v>
@@ -56320,7 +56332,7 @@
         <v>2772</v>
       </c>
       <c r="H22" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I22">
         <v>0</v>
@@ -56409,7 +56421,7 @@
         <v>4288</v>
       </c>
       <c r="H23" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I23">
         <v>0</v>
@@ -56587,7 +56599,7 @@
         <v>2957</v>
       </c>
       <c r="H25" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I25">
         <v>0</v>
@@ -56851,7 +56863,7 @@
         <v>2332</v>
       </c>
       <c r="H28" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I28">
         <v>100000</v>
@@ -57032,7 +57044,7 @@
         <v>1848</v>
       </c>
       <c r="H30" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I30">
         <v>0</v>
@@ -57124,7 +57136,7 @@
         <v>2951</v>
       </c>
       <c r="H31" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I31">
         <v>0</v>
@@ -57391,7 +57403,7 @@
         <v>3103</v>
       </c>
       <c r="H34" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I34">
         <v>1400000</v>
@@ -57842,7 +57854,7 @@
         <v>3156</v>
       </c>
       <c r="H39" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I39">
         <v>0</v>
@@ -57931,7 +57943,7 @@
         <v>3313</v>
       </c>
       <c r="H40" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I40">
         <v>200000</v>
@@ -58290,7 +58302,7 @@
         <v>3143</v>
       </c>
       <c r="H44" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I44">
         <v>0</v>
@@ -58379,7 +58391,7 @@
         <v>2481</v>
       </c>
       <c r="H45" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I45">
         <v>1500000</v>
@@ -58468,7 +58480,7 @@
         <v>1643</v>
       </c>
       <c r="H46" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I46">
         <v>0</v>
@@ -58560,7 +58572,7 @@
         <v>1569</v>
       </c>
       <c r="H47" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I47">
         <v>250000</v>
@@ -58649,7 +58661,7 @@
         <v>1413</v>
       </c>
       <c r="H48" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I48">
         <v>0</v>
@@ -58830,7 +58842,7 @@
         <v>1878</v>
       </c>
       <c r="H50" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I50">
         <v>300000</v>
@@ -59094,7 +59106,7 @@
         <v>2215</v>
       </c>
       <c r="H53" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I53">
         <v>0</v>
@@ -59361,7 +59373,7 @@
         <v>1913</v>
       </c>
       <c r="H56" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I56">
         <v>0</v>
@@ -60438,7 +60450,7 @@
         <v>3285</v>
       </c>
       <c r="H68" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I68">
         <v>1200000</v>
@@ -60619,7 +60631,7 @@
         <v>3030</v>
       </c>
       <c r="H70" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I70">
         <v>0</v>
@@ -60708,7 +60720,7 @@
         <v>2937</v>
       </c>
       <c r="H71" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I71">
         <v>0</v>
@@ -60797,7 +60809,7 @@
         <v>3446</v>
       </c>
       <c r="H72" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I72">
         <v>1200000</v>
@@ -60889,7 +60901,7 @@
         <v>3753</v>
       </c>
       <c r="H73" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I73">
         <v>0</v>
@@ -60978,7 +60990,7 @@
         <v>2756</v>
       </c>
       <c r="H74" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I74">
         <v>0</v>
@@ -61334,7 +61346,7 @@
         <v>2744</v>
       </c>
       <c r="H78" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="I78">
         <v>0</v>
@@ -61423,7 +61435,7 @@
         <v>2655</v>
       </c>
       <c r="H79" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I79">
         <v>1000000</v>
@@ -61512,7 +61524,7 @@
         <v>2474</v>
       </c>
       <c r="H80" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I80">
         <v>0</v>
@@ -61957,7 +61969,7 @@
         <v>1349</v>
       </c>
       <c r="H85" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I85">
         <v>250000</v>
@@ -62049,7 +62061,7 @@
         <v>3057</v>
       </c>
       <c r="H86" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I86">
         <v>800000</v>
@@ -62230,7 +62242,7 @@
         <v>3287</v>
       </c>
       <c r="H88" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I88">
         <v>400000</v>
@@ -62592,7 +62604,7 @@
         <v>2016</v>
       </c>
       <c r="H92" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I92">
         <v>0</v>
@@ -62859,7 +62871,7 @@
         <v>2642</v>
       </c>
       <c r="H95" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I95">
         <v>800000</v>
@@ -62951,7 +62963,7 @@
         <v>1747</v>
       </c>
       <c r="H96" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I96">
         <v>500000</v>
@@ -63043,7 +63055,7 @@
         <v>2146</v>
       </c>
       <c r="H97" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I97">
         <v>0</v>
@@ -63663,7 +63675,7 @@
         <v>2658</v>
       </c>
       <c r="H104" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I104">
         <v>1500000</v>
@@ -63752,7 +63764,7 @@
         <v>1802</v>
       </c>
       <c r="H105" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I105">
         <v>0</v>
@@ -63841,7 +63853,7 @@
         <v>2415</v>
       </c>
       <c r="H106" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I106">
         <v>0</v>
@@ -64111,7 +64123,7 @@
         <v>2176</v>
       </c>
       <c r="H109" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I109">
         <v>0</v>
@@ -64200,7 +64212,7 @@
         <v>2142</v>
       </c>
       <c r="H110" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I110">
         <v>0</v>
@@ -67003,7 +67015,7 @@
         <v>996</v>
       </c>
       <c r="H26" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="I26">
         <v>600000</v>
@@ -89730,7 +89742,7 @@
         <v>1087</v>
       </c>
       <c r="H246" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J246" t="s">
         <v>272</v>

</xml_diff>

<commit_message>
Série A: mais 6 vetos (Gabriel Mec, Herrera, Italo, J. Rojas, Pedro Gabriel, Tiago Volpi)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EuPBN7B2QoMn8WDwKax4KN
</commit_message>
<xml_diff>
--- a/Santa Cruz V2/listas/listas_2027.xlsx
+++ b/Santa Cruz V2/listas/listas_2027.xlsx
@@ -907,9 +907,6 @@
     <t>Ronaldo</t>
   </si>
   <si>
-    <t>Tiago Volpi</t>
-  </si>
-  <si>
     <t>Lucas Arcanjo</t>
   </si>
   <si>
@@ -928,6 +925,9 @@
     <t>Rafael</t>
   </si>
   <si>
+    <t>Hugo Souza</t>
+  </si>
+  <si>
     <t>Lucas Ramon</t>
   </si>
   <si>
@@ -1102,12 +1102,12 @@
     <t>Gabriel Bontempo</t>
   </si>
   <si>
-    <t>J. Herrera</t>
-  </si>
-  <si>
     <t>Nuno Moreira</t>
   </si>
   <si>
+    <t>J. Enamorado</t>
+  </si>
+  <si>
     <t>Samuel Lino</t>
   </si>
   <si>
@@ -1156,27 +1156,30 @@
     <t>Bahia</t>
   </si>
   <si>
+    <t>Vitória</t>
+  </si>
+  <si>
+    <t>Athletico Paranaense</t>
+  </si>
+  <si>
+    <t>Coritiba</t>
+  </si>
+  <si>
+    <t>Atlético Mineiro</t>
+  </si>
+  <si>
+    <t>São Paulo</t>
+  </si>
+  <si>
+    <t>Corinthians</t>
+  </si>
+  <si>
+    <t>Remo</t>
+  </si>
+  <si>
     <t>Red Bull Bragantino</t>
   </si>
   <si>
-    <t>Vitória</t>
-  </si>
-  <si>
-    <t>Athletico Paranaense</t>
-  </si>
-  <si>
-    <t>Coritiba</t>
-  </si>
-  <si>
-    <t>Atlético Mineiro</t>
-  </si>
-  <si>
-    <t>São Paulo</t>
-  </si>
-  <si>
-    <t>Remo</t>
-  </si>
-  <si>
     <t>Palmeiras</t>
   </si>
   <si>
@@ -1187,9 +1190,6 @@
   </si>
   <si>
     <t>Cruzeiro</t>
-  </si>
-  <si>
-    <t>Corinthians</t>
   </si>
   <si>
     <t>Mirassol</t>
@@ -22548,16 +22548,16 @@
         <v>378</v>
       </c>
       <c r="F3">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="G3">
-        <v>1534</v>
+        <v>1963</v>
       </c>
       <c r="H3" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="I3">
-        <v>1500000</v>
+        <v>1000000</v>
       </c>
       <c r="J3" t="s">
         <v>272</v>
@@ -22566,19 +22566,19 @@
         <v>272</v>
       </c>
       <c r="L3">
-        <v>70.5</v>
+        <v>53.4</v>
       </c>
       <c r="M3">
-        <v>67.7</v>
+        <v>63</v>
       </c>
       <c r="N3">
-        <v>71.09999999999999</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="O3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="P3">
-        <v>69.40000000000001</v>
+        <v>64</v>
       </c>
       <c r="Q3" t="b">
         <v>1</v>
@@ -22590,13 +22590,13 @@
         <v>5</v>
       </c>
       <c r="U3">
-        <v>45.2</v>
+        <v>43.4</v>
       </c>
       <c r="V3">
         <v>0.1</v>
       </c>
       <c r="W3">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="X3">
         <v>0.1</v>
@@ -22611,7 +22611,7 @@
         <v>284</v>
       </c>
       <c r="AB3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC3" t="b">
         <v>0</v>
@@ -22637,13 +22637,13 @@
         <v>379</v>
       </c>
       <c r="F4">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="G4">
-        <v>1963</v>
+        <v>2256</v>
       </c>
       <c r="H4" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="I4">
         <v>1000000</v>
@@ -22655,19 +22655,19 @@
         <v>272</v>
       </c>
       <c r="L4">
-        <v>53.4</v>
+        <v>48.3</v>
       </c>
       <c r="M4">
-        <v>63</v>
+        <v>61.5</v>
       </c>
       <c r="N4">
-        <v>64.90000000000001</v>
+        <v>58.4</v>
       </c>
       <c r="O4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P4">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="Q4" t="b">
         <v>1</v>
@@ -22679,13 +22679,13 @@
         <v>5</v>
       </c>
       <c r="U4">
-        <v>43.4</v>
+        <v>46.8</v>
       </c>
       <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
         <v>0.1</v>
-      </c>
-      <c r="W4">
-        <v>0.2</v>
       </c>
       <c r="X4">
         <v>0.1</v>
@@ -22700,7 +22700,7 @@
         <v>284</v>
       </c>
       <c r="AB4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC4" t="b">
         <v>0</v>
@@ -22723,19 +22723,19 @@
         <v>297</v>
       </c>
       <c r="E5" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="F5">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G5">
-        <v>2256</v>
+        <v>1584</v>
       </c>
       <c r="H5" t="s">
         <v>253</v>
       </c>
       <c r="I5">
-        <v>1000000</v>
+        <v>100000</v>
       </c>
       <c r="J5" t="s">
         <v>272</v>
@@ -22744,19 +22744,19 @@
         <v>272</v>
       </c>
       <c r="L5">
-        <v>48.3</v>
+        <v>65.3</v>
       </c>
       <c r="M5">
-        <v>61.5</v>
+        <v>66.3</v>
       </c>
       <c r="N5">
-        <v>58.4</v>
+        <v>49.9</v>
       </c>
       <c r="O5">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="P5">
-        <v>60</v>
+        <v>58.1</v>
       </c>
       <c r="Q5" t="b">
         <v>1</v>
@@ -22768,13 +22768,13 @@
         <v>5</v>
       </c>
       <c r="U5">
-        <v>46.8</v>
+        <v>51.6</v>
       </c>
       <c r="V5">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="W5">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="X5">
         <v>0.1</v>
@@ -22812,19 +22812,19 @@
         <v>298</v>
       </c>
       <c r="E6" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="F6">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="G6">
-        <v>1584</v>
+        <v>1623</v>
       </c>
       <c r="H6" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="I6">
-        <v>100000</v>
+        <v>600000</v>
       </c>
       <c r="J6" t="s">
         <v>272</v>
@@ -22833,19 +22833,19 @@
         <v>272</v>
       </c>
       <c r="L6">
-        <v>65.3</v>
+        <v>56.8</v>
       </c>
       <c r="M6">
-        <v>66.3</v>
+        <v>63.9</v>
       </c>
       <c r="N6">
-        <v>49.9</v>
+        <v>50.9</v>
       </c>
       <c r="O6">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P6">
-        <v>58.1</v>
+        <v>57.4</v>
       </c>
       <c r="Q6" t="b">
         <v>1</v>
@@ -22857,13 +22857,13 @@
         <v>5</v>
       </c>
       <c r="U6">
-        <v>51.6</v>
+        <v>39.5</v>
       </c>
       <c r="V6">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="W6">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="X6">
         <v>0.1</v>
@@ -22878,7 +22878,7 @@
         <v>284</v>
       </c>
       <c r="AB6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC6" t="b">
         <v>0</v>
@@ -22904,16 +22904,16 @@
         <v>381</v>
       </c>
       <c r="F7">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="G7">
-        <v>1623</v>
+        <v>2201</v>
       </c>
       <c r="H7" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="I7">
-        <v>600000</v>
+        <v>1800000</v>
       </c>
       <c r="J7" t="s">
         <v>272</v>
@@ -22922,19 +22922,19 @@
         <v>272</v>
       </c>
       <c r="L7">
-        <v>56.8</v>
+        <v>48.9</v>
       </c>
       <c r="M7">
-        <v>63.9</v>
+        <v>61.7</v>
       </c>
       <c r="N7">
-        <v>50.9</v>
+        <v>50.8</v>
       </c>
       <c r="O7">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P7">
-        <v>57.4</v>
+        <v>56.3</v>
       </c>
       <c r="Q7" t="b">
         <v>1</v>
@@ -22946,16 +22946,16 @@
         <v>5</v>
       </c>
       <c r="U7">
-        <v>39.5</v>
+        <v>49.3</v>
       </c>
       <c r="V7">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="W7">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="X7">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="Y7" t="b">
         <v>1</v>
@@ -22993,16 +22993,16 @@
         <v>382</v>
       </c>
       <c r="F8">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G8">
-        <v>2201</v>
+        <v>2265</v>
       </c>
       <c r="H8" t="s">
         <v>256</v>
       </c>
       <c r="I8">
-        <v>1800000</v>
+        <v>800000</v>
       </c>
       <c r="J8" t="s">
         <v>272</v>
@@ -23011,7 +23011,7 @@
         <v>272</v>
       </c>
       <c r="L8">
-        <v>48.9</v>
+        <v>49.1</v>
       </c>
       <c r="M8">
         <v>61.7</v>
@@ -23020,10 +23020,10 @@
         <v>50.8</v>
       </c>
       <c r="O8">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P8">
-        <v>56.3</v>
+        <v>56.2</v>
       </c>
       <c r="Q8" t="b">
         <v>1</v>
@@ -23035,16 +23035,16 @@
         <v>5</v>
       </c>
       <c r="U8">
-        <v>49.3</v>
+        <v>53.8</v>
       </c>
       <c r="V8">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="W8">
         <v>0.3</v>
       </c>
       <c r="X8">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="Y8" t="b">
         <v>1</v>
@@ -23082,16 +23082,16 @@
         <v>383</v>
       </c>
       <c r="F9">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="G9">
-        <v>2265</v>
+        <v>2160</v>
       </c>
       <c r="H9" t="s">
-        <v>256</v>
+        <v>396</v>
       </c>
       <c r="I9">
-        <v>800000</v>
+        <v>0</v>
       </c>
       <c r="J9" t="s">
         <v>272</v>
@@ -23100,19 +23100,19 @@
         <v>272</v>
       </c>
       <c r="L9">
-        <v>49.1</v>
+        <v>36.4</v>
       </c>
       <c r="M9">
-        <v>61.7</v>
+        <v>58.2</v>
       </c>
       <c r="N9">
-        <v>50.8</v>
+        <v>52.6</v>
       </c>
       <c r="O9">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="P9">
-        <v>56.2</v>
+        <v>55.4</v>
       </c>
       <c r="Q9" t="b">
         <v>1</v>
@@ -23124,13 +23124,13 @@
         <v>5</v>
       </c>
       <c r="U9">
-        <v>53.8</v>
+        <v>51</v>
       </c>
       <c r="V9">
         <v>0.1</v>
       </c>
       <c r="W9">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="X9">
         <v>0.1</v>
@@ -23168,7 +23168,7 @@
         <v>302</v>
       </c>
       <c r="E10" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="F10">
         <v>32</v>
@@ -23349,7 +23349,7 @@
         <v>304</v>
       </c>
       <c r="E12" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="F12">
         <v>24</v>
@@ -23441,7 +23441,7 @@
         <v>305</v>
       </c>
       <c r="E13" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F13">
         <v>30</v>
@@ -23533,7 +23533,7 @@
         <v>306</v>
       </c>
       <c r="E14" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F14">
         <v>22</v>
@@ -23625,7 +23625,7 @@
         <v>307</v>
       </c>
       <c r="E15" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F15">
         <v>33</v>
@@ -23717,7 +23717,7 @@
         <v>308</v>
       </c>
       <c r="E16" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F16">
         <v>32</v>
@@ -23809,7 +23809,7 @@
         <v>309</v>
       </c>
       <c r="E17" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F17">
         <v>31</v>
@@ -23901,7 +23901,7 @@
         <v>310</v>
       </c>
       <c r="E18" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F18">
         <v>30</v>
@@ -24085,7 +24085,7 @@
         <v>312</v>
       </c>
       <c r="E20" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F20">
         <v>30</v>
@@ -24177,7 +24177,7 @@
         <v>313</v>
       </c>
       <c r="E21" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="F21">
         <v>26</v>
@@ -24269,7 +24269,7 @@
         <v>314</v>
       </c>
       <c r="E22" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="F22">
         <v>35</v>
@@ -24453,7 +24453,7 @@
         <v>316</v>
       </c>
       <c r="E24" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F24">
         <v>22</v>
@@ -24729,7 +24729,7 @@
         <v>319</v>
       </c>
       <c r="E27" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F27">
         <v>30</v>
@@ -24913,7 +24913,7 @@
         <v>321</v>
       </c>
       <c r="E29" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F29">
         <v>32</v>
@@ -25097,7 +25097,7 @@
         <v>323</v>
       </c>
       <c r="E31" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F31">
         <v>22</v>
@@ -25189,7 +25189,7 @@
         <v>324</v>
       </c>
       <c r="E32" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="F32">
         <v>29</v>
@@ -25281,7 +25281,7 @@
         <v>325</v>
       </c>
       <c r="E33" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F33">
         <v>27</v>
@@ -25465,7 +25465,7 @@
         <v>327</v>
       </c>
       <c r="E35" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F35">
         <v>34</v>
@@ -25557,7 +25557,7 @@
         <v>328</v>
       </c>
       <c r="E36" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="F36">
         <v>27</v>
@@ -25649,7 +25649,7 @@
         <v>329</v>
       </c>
       <c r="E37" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F37">
         <v>28</v>
@@ -25741,7 +25741,7 @@
         <v>330</v>
       </c>
       <c r="E38" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F38">
         <v>23</v>
@@ -26017,7 +26017,7 @@
         <v>333</v>
       </c>
       <c r="E41" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F41">
         <v>27</v>
@@ -26293,7 +26293,7 @@
         <v>162</v>
       </c>
       <c r="E44" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="F44">
         <v>31</v>
@@ -26569,7 +26569,7 @@
         <v>337</v>
       </c>
       <c r="E47" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F47">
         <v>26</v>
@@ -26741,7 +26741,7 @@
         <v>339</v>
       </c>
       <c r="E49" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F49">
         <v>29</v>
@@ -26821,7 +26821,7 @@
         <v>340</v>
       </c>
       <c r="E50" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="F50">
         <v>26</v>
@@ -27005,7 +27005,7 @@
         <v>342</v>
       </c>
       <c r="E52" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F52">
         <v>30</v>
@@ -27373,7 +27373,7 @@
         <v>345</v>
       </c>
       <c r="E56" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F56">
         <v>30</v>
@@ -27453,7 +27453,7 @@
         <v>346</v>
       </c>
       <c r="E57" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F57">
         <v>27</v>
@@ -27545,7 +27545,7 @@
         <v>347</v>
       </c>
       <c r="E58" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F58">
         <v>32</v>
@@ -27729,7 +27729,7 @@
         <v>349</v>
       </c>
       <c r="E60" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F60">
         <v>30</v>
@@ -27821,7 +27821,7 @@
         <v>350</v>
       </c>
       <c r="E61" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F61">
         <v>35</v>
@@ -27913,7 +27913,7 @@
         <v>351</v>
       </c>
       <c r="E62" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="F62">
         <v>28</v>
@@ -28005,7 +28005,7 @@
         <v>352</v>
       </c>
       <c r="E63" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="F63">
         <v>25</v>
@@ -28097,7 +28097,7 @@
         <v>192</v>
       </c>
       <c r="E64" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F64">
         <v>22</v>
@@ -28281,7 +28281,7 @@
         <v>354</v>
       </c>
       <c r="E66" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F66">
         <v>20</v>
@@ -28373,7 +28373,7 @@
         <v>355</v>
       </c>
       <c r="E67" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F67">
         <v>28</v>
@@ -28465,7 +28465,7 @@
         <v>356</v>
       </c>
       <c r="E68" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F68">
         <v>21</v>
@@ -28557,7 +28557,7 @@
         <v>357</v>
       </c>
       <c r="E69" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F69">
         <v>22</v>
@@ -28649,7 +28649,7 @@
         <v>358</v>
       </c>
       <c r="E70" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F70">
         <v>28</v>
@@ -28729,7 +28729,7 @@
         <v>359</v>
       </c>
       <c r="E71" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F71">
         <v>21</v>
@@ -28821,40 +28821,40 @@
         <v>360</v>
       </c>
       <c r="E72" t="s">
-        <v>378</v>
+        <v>394</v>
       </c>
       <c r="F72">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G72">
-        <v>1039</v>
+        <v>1005</v>
       </c>
       <c r="H72" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I72">
-        <v>0</v>
+        <v>1000000</v>
       </c>
       <c r="J72" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="K72" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="L72">
-        <v>62.7</v>
+        <v>34.5</v>
       </c>
       <c r="M72">
-        <v>65.59999999999999</v>
+        <v>57.7</v>
       </c>
       <c r="N72">
-        <v>43.8</v>
+        <v>50.2</v>
       </c>
       <c r="O72">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="P72">
-        <v>54.7</v>
+        <v>53.9</v>
       </c>
       <c r="Q72" t="b">
         <v>1</v>
@@ -28863,25 +28863,25 @@
         <v>0</v>
       </c>
       <c r="S72">
-        <v>43.5</v>
+        <v>36.9</v>
       </c>
       <c r="T72">
         <v>6</v>
       </c>
       <c r="U72">
-        <v>45.2</v>
+        <v>56.2</v>
       </c>
       <c r="V72">
-        <v>5.6</v>
+        <v>4.6</v>
       </c>
       <c r="W72">
-        <v>2.2</v>
+        <v>1.2</v>
       </c>
       <c r="X72">
-        <v>7.6</v>
+        <v>4.8</v>
       </c>
       <c r="Y72" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z72" t="b">
         <v>1</v>
@@ -28896,7 +28896,7 @@
         <v>0</v>
       </c>
       <c r="AD72" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="73" spans="1:30">
@@ -28913,40 +28913,40 @@
         <v>361</v>
       </c>
       <c r="E73" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="F73">
         <v>27</v>
       </c>
       <c r="G73">
-        <v>1005</v>
+        <v>975</v>
       </c>
       <c r="H73" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="I73">
-        <v>1000000</v>
+        <v>0</v>
       </c>
       <c r="J73" t="s">
-        <v>273</v>
+        <v>403</v>
       </c>
       <c r="K73" t="s">
-        <v>273</v>
+        <v>403</v>
       </c>
       <c r="L73">
-        <v>34.5</v>
+        <v>63.6</v>
       </c>
       <c r="M73">
-        <v>57.7</v>
+        <v>65.8</v>
       </c>
       <c r="N73">
-        <v>50.2</v>
+        <v>39.9</v>
       </c>
       <c r="O73">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="P73">
-        <v>53.9</v>
+        <v>52.8</v>
       </c>
       <c r="Q73" t="b">
         <v>1</v>
@@ -28955,25 +28955,25 @@
         <v>0</v>
       </c>
       <c r="S73">
-        <v>36.9</v>
+        <v>52.5</v>
       </c>
       <c r="T73">
         <v>6</v>
       </c>
       <c r="U73">
-        <v>56.2</v>
+        <v>48.3</v>
       </c>
       <c r="V73">
-        <v>4.6</v>
+        <v>6.3</v>
       </c>
       <c r="W73">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="X73">
-        <v>4.8</v>
+        <v>11.9</v>
       </c>
       <c r="Y73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z73" t="b">
         <v>1</v>
@@ -29005,7 +29005,7 @@
         <v>362</v>
       </c>
       <c r="E74" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F74">
         <v>26</v>
@@ -29189,7 +29189,7 @@
         <v>364</v>
       </c>
       <c r="E76" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="F76">
         <v>24</v>
@@ -29281,7 +29281,7 @@
         <v>365</v>
       </c>
       <c r="E77" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F77">
         <v>30</v>
@@ -29741,7 +29741,7 @@
         <v>370</v>
       </c>
       <c r="E82" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F82">
         <v>34</v>
@@ -29833,7 +29833,7 @@
         <v>371</v>
       </c>
       <c r="E83" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F83">
         <v>29</v>
@@ -29925,7 +29925,7 @@
         <v>372</v>
       </c>
       <c r="E84" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F84">
         <v>26</v>
@@ -30017,7 +30017,7 @@
         <v>373</v>
       </c>
       <c r="E85" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F85">
         <v>25</v>
@@ -30109,7 +30109,7 @@
         <v>374</v>
       </c>
       <c r="E86" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F86">
         <v>24</v>
@@ -30201,7 +30201,7 @@
         <v>331</v>
       </c>
       <c r="E87" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F87">
         <v>22</v>
@@ -30293,7 +30293,7 @@
         <v>375</v>
       </c>
       <c r="E88" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="F88">
         <v>34</v>
@@ -30385,7 +30385,7 @@
         <v>376</v>
       </c>
       <c r="E89" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F89">
         <v>26</v>

</xml_diff>